<commit_message>
refactor: force-override system prompt and preserve user message context
- Replace render_messages with build_messages that force-overrides system message content
- Remove Jinja2 dependency from dataset.py
- Save full user_content (with timestamps) in responses.jsonl for judge evaluation
- Fix evaluator.py to use user_content instead of query for judge messages
- Fix evaluator call signature bug: pass messages list directly, use model_copy for seed
- Update example.xlsx to use pure messages array format (no placeholders)

This enables datasets with hardcoded prompts to work seamlessly while maintaining
config/prompts as the single source of truth for system prompts.
</commit_message>
<xml_diff>
--- a/data/example.xlsx
+++ b/data/example.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>query</t>
   </si>
@@ -37,7 +37,19 @@
     <t>What is the difference between HTTP and HTTPS?</t>
   </si>
   <si>
-    <t>{"model": "PLACEHOLDER_MODEL", "messages": [{"role": "system", "content": "{{system_prompt}}"}, {"role": "user", "content": "{{query}}"}]}</t>
+    <t>[{"role": "system", "content": ""}, {"role": "user", "content": "[Current Time: 2024-06-01 14:30:00 CST] 什么是机器学习？"}]</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": ""}, {"role": "user", "content": "[Current Time: 2024-06-01 14:30:00 CST] Python中list和tuple的区别是什么？"}]</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": ""}, {"role": "user", "content": "[Current Time: 2024-06-01 14:30:00 CST] Explain the concept of recursion."}]</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": ""}, {"role": "user", "content": "[Current Time: 2024-06-01 14:30:00 CST] 如何用Docker部署一个Python应用？"}]</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": ""}, {"role": "user", "content": "[Current Time: 2024-06-01 14:30:00 CST] What is the difference between HTTP and HTTPS?"}]</t>
   </si>
 </sst>
 </file>
@@ -393,7 +405,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -401,7 +413,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -409,7 +421,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -417,7 +429,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>